<commit_message>
successful CRUD in Firestore and RTDB v9
</commit_message>
<xml_diff>
--- a/src/assets/data/materias.xlsx
+++ b/src/assets/data/materias.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="165">
   <si>
     <t xml:space="preserve">priority</t>
   </si>
@@ -37,6 +37,9 @@
     <t xml:space="preserve">description</t>
   </si>
   <si>
+    <t xml:space="preserve">cycle</t>
+  </si>
+  <si>
     <t xml:space="preserve">3° de Secundaria</t>
   </si>
   <si>
@@ -47,6 +50,9 @@
   </si>
   <si>
     <t xml:space="preserve">Curso de Español III de tipo Formativo para 3° de Secundaria.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CE20202021</t>
   </si>
   <si>
     <t xml:space="preserve">Matemáticas III</t>
@@ -518,7 +524,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -540,6 +546,12 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -584,7 +596,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -598,6 +610,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -618,14 +634,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E116"/>
-  <sheetFormatPr defaultColWidth="8.50390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F116"/>
+  <sheetFormatPr defaultColWidth="8.51171875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.03"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="42.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.69"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="77.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="23.2"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -644,22 +661,28 @@
       <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="0" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="F2" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -667,15 +690,18 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>10</v>
       </c>
     </row>
@@ -684,16 +710,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
+      </c>
+      <c r="F4" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -701,16 +730,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -718,16 +750,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
+      </c>
+      <c r="F6" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -735,16 +770,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -752,16 +790,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
+      </c>
+      <c r="F8" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -769,16 +810,19 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -786,16 +830,19 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
+      </c>
+      <c r="F10" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -803,16 +850,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -820,16 +870,19 @@
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C12" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>26</v>
-      </c>
       <c r="E12" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
+      </c>
+      <c r="F12" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -837,16 +890,19 @@
         <v>1</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -854,16 +910,19 @@
         <v>2</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
+      </c>
+      <c r="F14" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -871,16 +930,19 @@
         <v>3</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -888,16 +950,19 @@
         <v>4</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
+      </c>
+      <c r="F16" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -905,16 +970,19 @@
         <v>5</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -922,16 +990,19 @@
         <v>6</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>40</v>
+        <v>42</v>
+      </c>
+      <c r="F18" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -939,16 +1010,19 @@
         <v>7</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -956,16 +1030,19 @@
         <v>8</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
+      </c>
+      <c r="F20" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -973,16 +1050,19 @@
         <v>9</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -990,16 +1070,19 @@
         <v>10</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
+      </c>
+      <c r="F22" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1007,16 +1090,19 @@
         <v>11</v>
       </c>
       <c r="B23" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C23" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="D23" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D23" s="3" t="s">
-        <v>26</v>
-      </c>
       <c r="E23" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1024,16 +1110,19 @@
         <v>1</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
+      </c>
+      <c r="F24" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1041,16 +1130,19 @@
         <v>2</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1058,16 +1150,19 @@
         <v>3</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
+      </c>
+      <c r="F26" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1075,16 +1170,19 @@
         <v>4</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1092,16 +1190,19 @@
         <v>5</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
+      </c>
+      <c r="F28" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1109,16 +1210,19 @@
         <v>6</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1126,16 +1230,19 @@
         <v>7</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
+      </c>
+      <c r="F30" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1143,16 +1250,19 @@
         <v>8</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1160,16 +1270,19 @@
         <v>9</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
+      </c>
+      <c r="F32" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1177,16 +1290,19 @@
         <v>10</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1194,16 +1310,19 @@
         <v>11</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
+      </c>
+      <c r="F34" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1211,16 +1330,19 @@
         <v>12</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C35" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D35" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D35" s="3" t="s">
-        <v>26</v>
-      </c>
       <c r="E35" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1228,16 +1350,19 @@
         <v>1</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
+      </c>
+      <c r="F36" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1245,16 +1370,19 @@
         <v>2</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1262,16 +1390,19 @@
         <v>3</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
+      </c>
+      <c r="F38" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1279,16 +1410,19 @@
         <v>4</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1296,16 +1430,19 @@
         <v>5</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
+      </c>
+      <c r="F40" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1313,16 +1450,19 @@
         <v>6</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1330,16 +1470,19 @@
         <v>7</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
+      </c>
+      <c r="F42" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1347,16 +1490,19 @@
         <v>8</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1364,16 +1510,19 @@
         <v>9</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
+      </c>
+      <c r="F44" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1381,16 +1530,19 @@
         <v>10</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1398,16 +1550,19 @@
         <v>11</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
+      </c>
+      <c r="F46" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1415,16 +1570,19 @@
         <v>1</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1432,16 +1590,19 @@
         <v>2</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
+      </c>
+      <c r="F48" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1449,16 +1610,19 @@
         <v>3</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1466,16 +1630,19 @@
         <v>4</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
+      </c>
+      <c r="F50" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1483,16 +1650,19 @@
         <v>5</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1500,16 +1670,19 @@
         <v>6</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
+      </c>
+      <c r="F52" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1517,16 +1690,19 @@
         <v>7</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1534,16 +1710,19 @@
         <v>8</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
+      </c>
+      <c r="F54" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1551,16 +1730,19 @@
         <v>9</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1568,16 +1750,19 @@
         <v>10</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
+      </c>
+      <c r="F56" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1585,16 +1770,19 @@
         <v>11</v>
       </c>
       <c r="B57" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C57" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C57" s="3" t="s">
-        <v>75</v>
-      </c>
       <c r="D57" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1602,16 +1790,19 @@
         <v>1</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
+      </c>
+      <c r="F58" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1619,16 +1810,19 @@
         <v>2</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1636,16 +1830,19 @@
         <v>3</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
+      </c>
+      <c r="F60" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1653,16 +1850,19 @@
         <v>4</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
+      </c>
+      <c r="F61" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1670,16 +1870,19 @@
         <v>5</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
+      </c>
+      <c r="F62" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1687,16 +1890,19 @@
         <v>6</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
+      </c>
+      <c r="F63" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1704,16 +1910,19 @@
         <v>7</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
+      </c>
+      <c r="F64" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1721,16 +1930,19 @@
         <v>8</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
+      </c>
+      <c r="F65" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1738,16 +1950,19 @@
         <v>9</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
+      </c>
+      <c r="F66" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1755,16 +1970,19 @@
         <v>10</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1772,16 +1990,19 @@
         <v>11</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
+      </c>
+      <c r="F68" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1789,16 +2010,19 @@
         <v>1</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
+      </c>
+      <c r="F69" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1806,16 +2030,19 @@
         <v>2</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
+      </c>
+      <c r="F70" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1823,16 +2050,19 @@
         <v>3</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>104</v>
+        <v>106</v>
+      </c>
+      <c r="F71" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1840,16 +2070,19 @@
         <v>4</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
+      </c>
+      <c r="F72" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1857,16 +2090,19 @@
         <v>5</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
+      </c>
+      <c r="F73" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1874,16 +2110,19 @@
         <v>6</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
+      </c>
+      <c r="F74" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1891,16 +2130,19 @@
         <v>7</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1908,16 +2150,19 @@
         <v>8</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E76" s="3" t="s">
-        <v>110</v>
+        <v>112</v>
+      </c>
+      <c r="F76" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1925,16 +2170,19 @@
         <v>9</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>111</v>
+        <v>113</v>
+      </c>
+      <c r="F77" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1942,16 +2190,19 @@
         <v>10</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>112</v>
+        <v>114</v>
+      </c>
+      <c r="F78" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1959,16 +2210,19 @@
         <v>1</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>114</v>
+        <v>116</v>
+      </c>
+      <c r="F79" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1976,16 +2230,19 @@
         <v>2</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E80" s="3" t="s">
-        <v>115</v>
+        <v>117</v>
+      </c>
+      <c r="F80" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1993,16 +2250,19 @@
         <v>3</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E81" s="3" t="s">
-        <v>116</v>
+        <v>118</v>
+      </c>
+      <c r="F81" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2010,16 +2270,19 @@
         <v>4</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E82" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
+      </c>
+      <c r="F82" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2027,16 +2290,19 @@
         <v>5</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E83" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
+      </c>
+      <c r="F83" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2044,16 +2310,19 @@
         <v>6</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E84" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
+      </c>
+      <c r="F84" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2061,16 +2330,19 @@
         <v>7</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E85" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2078,16 +2350,19 @@
         <v>8</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E86" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
+      </c>
+      <c r="F86" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2095,16 +2370,19 @@
         <v>1</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>126</v>
+        <v>128</v>
+      </c>
+      <c r="F87" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2112,16 +2390,19 @@
         <v>2</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
+      </c>
+      <c r="F88" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2129,16 +2410,19 @@
         <v>3</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E89" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
+      </c>
+      <c r="F89" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2146,16 +2430,19 @@
         <v>4</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E90" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
+      </c>
+      <c r="F90" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2163,16 +2450,19 @@
         <v>5</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E91" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
+      </c>
+      <c r="F91" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2180,16 +2470,19 @@
         <v>6</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D92" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E92" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
+      </c>
+      <c r="F92" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2197,16 +2490,19 @@
         <v>7</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E93" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
+      </c>
+      <c r="F93" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2214,16 +2510,19 @@
         <v>8</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E94" s="3" t="s">
-        <v>133</v>
+        <v>135</v>
+      </c>
+      <c r="F94" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2231,16 +2530,19 @@
         <v>9</v>
       </c>
       <c r="B95" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C95" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="C95" s="3" t="s">
-        <v>123</v>
-      </c>
       <c r="D95" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E95" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
+      </c>
+      <c r="F95" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2248,16 +2550,19 @@
         <v>1</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E96" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
+      </c>
+      <c r="F96" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2265,16 +2570,19 @@
         <v>2</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E97" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
+      </c>
+      <c r="F97" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2282,16 +2590,19 @@
         <v>3</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D98" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E98" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
+      </c>
+      <c r="F98" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2299,16 +2610,19 @@
         <v>4</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D99" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E99" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
+      </c>
+      <c r="F99" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2316,16 +2630,19 @@
         <v>5</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D100" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E100" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
+      </c>
+      <c r="F100" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2333,16 +2650,19 @@
         <v>6</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D101" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E101" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
+      </c>
+      <c r="F101" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2350,16 +2670,19 @@
         <v>7</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D102" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E102" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
+      </c>
+      <c r="F102" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2367,16 +2690,19 @@
         <v>1</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D103" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E103" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
+      </c>
+      <c r="F103" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2384,16 +2710,19 @@
         <v>2</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D104" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E104" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
+      </c>
+      <c r="F104" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2401,16 +2730,19 @@
         <v>3</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D105" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E105" s="3" t="s">
-        <v>150</v>
+        <v>152</v>
+      </c>
+      <c r="F105" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2418,16 +2750,19 @@
         <v>4</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D106" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E106" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
+      </c>
+      <c r="F106" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2435,16 +2770,19 @@
         <v>5</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D107" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E107" s="3" t="s">
-        <v>152</v>
+        <v>154</v>
+      </c>
+      <c r="F107" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2452,16 +2790,19 @@
         <v>6</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D108" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E108" s="3" t="s">
-        <v>153</v>
+        <v>155</v>
+      </c>
+      <c r="F108" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2469,16 +2810,19 @@
         <v>7</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D109" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E109" s="3" t="s">
-        <v>154</v>
+        <v>156</v>
+      </c>
+      <c r="F109" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2486,16 +2830,19 @@
         <v>1</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D110" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E110" s="3" t="s">
-        <v>156</v>
+        <v>158</v>
+      </c>
+      <c r="F110" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2503,16 +2850,19 @@
         <v>2</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D111" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E111" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
+      </c>
+      <c r="F111" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2520,16 +2870,19 @@
         <v>3</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D112" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E112" s="3" t="s">
-        <v>158</v>
+        <v>160</v>
+      </c>
+      <c r="F112" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2537,16 +2890,19 @@
         <v>4</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D113" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E113" s="3" t="s">
-        <v>159</v>
+        <v>161</v>
+      </c>
+      <c r="F113" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2554,16 +2910,19 @@
         <v>5</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D114" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E114" s="3" t="s">
-        <v>160</v>
+        <v>162</v>
+      </c>
+      <c r="F114" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2571,16 +2930,19 @@
         <v>6</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D115" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E115" s="3" t="s">
-        <v>161</v>
+        <v>163</v>
+      </c>
+      <c r="F115" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2588,16 +2950,19 @@
         <v>7</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D116" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E116" s="3" t="s">
-        <v>162</v>
+        <v>164</v>
+      </c>
+      <c r="F116" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
comine classrooms and courses by id done
</commit_message>
<xml_diff>
--- a/src/assets/data/materias.xlsx
+++ b/src/assets/data/materias.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet1!$A$1:$G$231</definedName>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet1!$B$1:$H$231</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet1!$A$1:$G$231</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm._FilterDatabase_0" vbProcedure="false">Sheet1!$B$1:$H$231</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -253,7 +253,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="4">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -275,20 +275,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <u val="single"/>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -333,7 +319,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -366,14 +352,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -386,17 +364,13 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="true">
+  <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H233"/>
-  <sheetFormatPr defaultColWidth="8.5625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:H1048576"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="27.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="7.26"/>
@@ -431,7 +405,7 @@
       </c>
       <c r="H1" s="3"/>
     </row>
-    <row r="2" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
@@ -462,7 +436,7 @@
       <c r="B3" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="3" t="s">
@@ -479,14 +453,14 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="3" t="s">
@@ -503,14 +477,14 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D5" s="3" t="s">
@@ -527,14 +501,14 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D6" s="3" t="s">
@@ -551,14 +525,14 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D7" s="3" t="s">
@@ -575,14 +549,14 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D8" s="3" t="s">
@@ -599,14 +573,14 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D9" s="3" t="s">
@@ -623,14 +597,14 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="3" t="s">
         <v>25</v>
       </c>
       <c r="D10" s="3" t="s">
@@ -647,7 +621,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
         <v>27</v>
       </c>
@@ -671,7 +645,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
         <v>27</v>
       </c>
@@ -695,7 +669,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
         <v>27</v>
       </c>
@@ -719,24 +693,24 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="1" t="n">
+      <c r="B14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="0" t="s">
+      <c r="D14" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E14" s="3" t="str">
         <f aca="false">_xlfn.CONCAT("Curso de ",A14," de tipo ",D14, " para ",C14," durante el ciclo escolar ", F14,".")</f>
         <v>Curso de Español III de tipo Formativo para SECUNDARIA_2 durante el ciclo escolar CE20212022.</v>
       </c>
-      <c r="F14" s="0" t="s">
+      <c r="F14" s="3" t="s">
         <v>33</v>
       </c>
       <c r="G14" s="2" t="s">
@@ -744,16 +718,16 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="1" t="n">
+      <c r="B15" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D15" s="0" t="s">
+      <c r="D15" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E15" s="3" t="str">
@@ -767,17 +741,17 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B16" s="1" t="n">
+      <c r="B16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D16" s="0" t="s">
+      <c r="D16" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E16" s="3" t="str">
@@ -791,17 +765,17 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B17" s="1" t="n">
+      <c r="B17" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="C17" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D17" s="0" t="s">
+      <c r="D17" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E17" s="3" t="str">
@@ -815,17 +789,17 @@
         <v>34</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="1" t="n">
+      <c r="B18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="C18" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D18" s="0" t="s">
+      <c r="D18" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E18" s="3" t="str">
@@ -839,17 +813,17 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="1" t="n">
+      <c r="B19" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D19" s="0" t="s">
+      <c r="D19" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E19" s="3" t="str">
@@ -863,17 +837,17 @@
         <v>22</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B20" s="1" t="n">
+      <c r="B20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="C20" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D20" s="0" t="s">
+      <c r="D20" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E20" s="3" t="str">
@@ -887,17 +861,17 @@
         <v>16</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B21" s="1" t="n">
+      <c r="B21" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="C21" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D21" s="0" t="s">
+      <c r="D21" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E21" s="3" t="str">
@@ -911,17 +885,17 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B22" s="1" t="n">
+      <c r="B22" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C22" s="0" t="s">
+      <c r="C22" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D22" s="0" t="s">
+      <c r="D22" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E22" s="3" t="str">
@@ -935,17 +909,17 @@
         <v>26</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="1" t="n">
+      <c r="B23" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D23" s="0" t="s">
+      <c r="D23" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E23" s="3" t="str">
@@ -959,17 +933,17 @@
         <v>29</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B24" s="1" t="n">
+      <c r="B24" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D24" s="0" t="s">
+      <c r="D24" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E24" s="3" t="str">
@@ -983,17 +957,17 @@
         <v>31</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B25" s="1" t="n">
+      <c r="B25" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C25" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D25" s="0" t="s">
+      <c r="D25" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E25" s="3" t="str">
@@ -1007,7 +981,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
         <v>35</v>
       </c>
@@ -1038,7 +1012,7 @@
       <c r="B27" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D27" s="3" t="s">
@@ -1055,14 +1029,14 @@
         <v>36</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B28" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C28" s="0" t="s">
+      <c r="C28" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D28" s="3" t="s">
@@ -1079,14 +1053,14 @@
         <v>36</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B29" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C29" s="0" t="s">
+      <c r="C29" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D29" s="3" t="s">
@@ -1103,14 +1077,14 @@
         <v>16</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B30" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C30" s="0" t="s">
+      <c r="C30" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D30" s="3" t="s">
@@ -1127,14 +1101,14 @@
         <v>18</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B31" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C31" s="8" t="s">
+      <c r="C31" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D31" s="3" t="s">
@@ -1151,14 +1125,14 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B32" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C32" s="0" t="s">
+      <c r="C32" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D32" s="3" t="s">
@@ -1175,14 +1149,14 @@
         <v>22</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B33" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C33" s="0" t="s">
+      <c r="C33" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D33" s="3" t="s">
@@ -1199,14 +1173,14 @@
         <v>24</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B34" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C34" s="0" t="s">
+      <c r="C34" s="3" t="s">
         <v>25</v>
       </c>
       <c r="D34" s="3" t="s">
@@ -1223,7 +1197,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
         <v>38</v>
       </c>
@@ -1247,7 +1221,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
         <v>38</v>
       </c>
@@ -1271,7 +1245,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
         <v>38</v>
       </c>
@@ -1295,17 +1269,17 @@
         <v>39</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B38" s="1" t="n">
+      <c r="B38" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D38" s="0" t="s">
+      <c r="D38" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E38" s="3" t="str">
@@ -1320,16 +1294,16 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0" t="s">
+      <c r="A39" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B39" s="1" t="n">
+      <c r="B39" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C39" s="8" t="s">
+      <c r="C39" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D39" s="0" t="s">
+      <c r="D39" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E39" s="3" t="str">
@@ -1343,17 +1317,17 @@
         <v>36</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="0" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B40" s="1" t="n">
+      <c r="B40" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C40" s="0" t="s">
+      <c r="C40" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D40" s="0" t="s">
+      <c r="D40" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E40" s="3" t="str">
@@ -1367,17 +1341,17 @@
         <v>36</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="0" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B41" s="1" t="n">
+      <c r="B41" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C41" s="0" t="s">
+      <c r="C41" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D41" s="0" t="s">
+      <c r="D41" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E41" s="3" t="str">
@@ -1391,17 +1365,17 @@
         <v>34</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="0" t="s">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B42" s="1" t="n">
+      <c r="B42" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C42" s="0" t="s">
+      <c r="C42" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D42" s="0" t="s">
+      <c r="D42" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E42" s="3" t="str">
@@ -1415,17 +1389,17 @@
         <v>20</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="0" t="s">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B43" s="1" t="n">
+      <c r="B43" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C43" s="8" t="s">
+      <c r="C43" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D43" s="0" t="s">
+      <c r="D43" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E43" s="3" t="str">
@@ -1439,17 +1413,17 @@
         <v>22</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="0" t="s">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B44" s="1" t="n">
+      <c r="B44" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C44" s="0" t="s">
+      <c r="C44" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D44" s="0" t="s">
+      <c r="D44" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E44" s="3" t="str">
@@ -1463,17 +1437,17 @@
         <v>16</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="0" t="s">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B45" s="1" t="n">
+      <c r="B45" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C45" s="0" t="s">
+      <c r="C45" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D45" s="0" t="s">
+      <c r="D45" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E45" s="3" t="str">
@@ -1487,17 +1461,17 @@
         <v>24</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="0" t="s">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B46" s="1" t="n">
+      <c r="B46" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C46" s="0" t="s">
+      <c r="C46" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D46" s="0" t="s">
+      <c r="D46" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E46" s="3" t="str">
@@ -1511,17 +1485,17 @@
         <v>26</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="0" t="s">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B47" s="1" t="n">
+      <c r="B47" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D47" s="0" t="s">
+      <c r="D47" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E47" s="3" t="str">
@@ -1535,17 +1509,17 @@
         <v>40</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="0" t="s">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B48" s="1" t="n">
+      <c r="B48" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D48" s="0" t="s">
+      <c r="D48" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E48" s="3" t="str">
@@ -1559,17 +1533,17 @@
         <v>40</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="0" t="s">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B49" s="1" t="n">
+      <c r="B49" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="C49" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D49" s="0" t="s">
+      <c r="D49" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E49" s="3" t="str">
@@ -1583,7 +1557,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
         <v>41</v>
       </c>
@@ -1614,7 +1588,7 @@
       <c r="B51" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C51" s="8" t="s">
+      <c r="C51" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D51" s="3" t="s">
@@ -1631,14 +1605,14 @@
         <v>43</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
         <v>42</v>
       </c>
       <c r="B52" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C52" s="0" t="s">
+      <c r="C52" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D52" s="3" t="s">
@@ -1655,14 +1629,14 @@
         <v>43</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
         <v>42</v>
       </c>
       <c r="B53" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C53" s="0" t="s">
+      <c r="C53" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D53" s="3" t="s">
@@ -1679,14 +1653,14 @@
         <v>43</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
         <v>42</v>
       </c>
       <c r="B54" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C54" s="0" t="s">
+      <c r="C54" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D54" s="3" t="s">
@@ -1703,14 +1677,14 @@
         <v>43</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
         <v>42</v>
       </c>
       <c r="B55" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C55" s="8" t="s">
+      <c r="C55" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D55" s="3" t="s">
@@ -1727,14 +1701,14 @@
         <v>43</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
         <v>42</v>
       </c>
       <c r="B56" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C56" s="0" t="s">
+      <c r="C56" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D56" s="3" t="s">
@@ -1751,14 +1725,14 @@
         <v>44</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
         <v>42</v>
       </c>
       <c r="B57" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C57" s="0" t="s">
+      <c r="C57" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D57" s="3" t="s">
@@ -1775,14 +1749,14 @@
         <v>44</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
         <v>42</v>
       </c>
       <c r="B58" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C58" s="0" t="s">
+      <c r="C58" s="3" t="s">
         <v>25</v>
       </c>
       <c r="D58" s="3" t="s">
@@ -1799,7 +1773,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
         <v>45</v>
       </c>
@@ -1823,7 +1797,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
         <v>45</v>
       </c>
@@ -1847,14 +1821,14 @@
         <v>31</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
         <v>45</v>
       </c>
       <c r="B61" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C61" s="9" t="s">
+      <c r="C61" s="3" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="3" t="s">
@@ -1871,17 +1845,17 @@
         <v>31</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="0" t="s">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B62" s="1" t="n">
+      <c r="B62" s="4" t="n">
         <v>3</v>
       </c>
       <c r="C62" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D62" s="0" t="s">
+      <c r="D62" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E62" s="3" t="str">
@@ -1896,16 +1870,16 @@
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="0" t="s">
+      <c r="A63" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B63" s="1" t="n">
+      <c r="B63" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C63" s="8" t="s">
+      <c r="C63" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D63" s="0" t="s">
+      <c r="D63" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E63" s="3" t="str">
@@ -1919,17 +1893,17 @@
         <v>40</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="0" t="s">
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B64" s="1" t="n">
+      <c r="B64" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C64" s="0" t="s">
+      <c r="C64" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D64" s="0" t="s">
+      <c r="D64" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E64" s="3" t="str">
@@ -1943,17 +1917,17 @@
         <v>40</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="0" t="s">
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B65" s="1" t="n">
+      <c r="B65" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C65" s="0" t="s">
+      <c r="C65" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D65" s="0" t="s">
+      <c r="D65" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E65" s="3" t="str">
@@ -1967,17 +1941,17 @@
         <v>43</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="0" t="s">
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B66" s="1" t="n">
+      <c r="B66" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C66" s="0" t="s">
+      <c r="C66" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D66" s="0" t="s">
+      <c r="D66" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E66" s="3" t="str">
@@ -1991,17 +1965,17 @@
         <v>43</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="0" t="s">
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B67" s="1" t="n">
+      <c r="B67" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C67" s="8" t="s">
+      <c r="C67" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D67" s="0" t="s">
+      <c r="D67" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E67" s="3" t="str">
@@ -2015,17 +1989,17 @@
         <v>43</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="0" t="s">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B68" s="1" t="n">
+      <c r="B68" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C68" s="0" t="s">
+      <c r="C68" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D68" s="0" t="s">
+      <c r="D68" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E68" s="3" t="str">
@@ -2039,17 +2013,17 @@
         <v>44</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="0" t="s">
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B69" s="1" t="n">
+      <c r="B69" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C69" s="0" t="s">
+      <c r="C69" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D69" s="0" t="s">
+      <c r="D69" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E69" s="3" t="str">
@@ -2063,17 +2037,17 @@
         <v>44</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="0" t="s">
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B70" s="1" t="n">
+      <c r="B70" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C70" s="0" t="s">
+      <c r="C70" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D70" s="0" t="s">
+      <c r="D70" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E70" s="3" t="str">
@@ -2087,17 +2061,17 @@
         <v>44</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="0" t="s">
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B71" s="1" t="n">
+      <c r="B71" s="4" t="n">
         <v>3</v>
       </c>
       <c r="C71" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D71" s="0" t="s">
+      <c r="D71" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E71" s="3" t="str">
@@ -2111,17 +2085,17 @@
         <v>29</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="0" t="s">
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B72" s="1" t="n">
+      <c r="B72" s="4" t="n">
         <v>3</v>
       </c>
       <c r="C72" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D72" s="0" t="s">
+      <c r="D72" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E72" s="3" t="str">
@@ -2135,17 +2109,17 @@
         <v>31</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="0" t="s">
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B73" s="1" t="n">
+      <c r="B73" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C73" s="9" t="s">
+      <c r="C73" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D73" s="0" t="s">
+      <c r="D73" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E73" s="3" t="str">
@@ -2159,7 +2133,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
         <v>46</v>
       </c>
@@ -2190,7 +2164,7 @@
       <c r="B75" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C75" s="8" t="s">
+      <c r="C75" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D75" s="3" t="s">
@@ -2207,14 +2181,14 @@
         <v>36</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
         <v>49</v>
       </c>
       <c r="B76" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C76" s="0" t="s">
+      <c r="C76" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D76" s="3" t="s">
@@ -2231,14 +2205,14 @@
         <v>50</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="3" t="s">
         <v>51</v>
       </c>
       <c r="B77" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C77" s="0" t="s">
+      <c r="C77" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D77" s="3" t="s">
@@ -2255,14 +2229,14 @@
         <v>16</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
         <v>51</v>
       </c>
       <c r="B78" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C78" s="0" t="s">
+      <c r="C78" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D78" s="3" t="s">
@@ -2279,14 +2253,14 @@
         <v>18</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="3" t="s">
         <v>51</v>
       </c>
       <c r="B79" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C79" s="8" t="s">
+      <c r="C79" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D79" s="3" t="s">
@@ -2303,14 +2277,14 @@
         <v>20</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="3" t="s">
         <v>51</v>
       </c>
       <c r="B80" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C80" s="0" t="s">
+      <c r="C80" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D80" s="3" t="s">
@@ -2327,14 +2301,14 @@
         <v>22</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="3" t="s">
         <v>52</v>
       </c>
       <c r="B81" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C81" s="0" t="s">
+      <c r="C81" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D81" s="3" t="s">
@@ -2351,14 +2325,14 @@
         <v>24</v>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="3" t="s">
         <v>52</v>
       </c>
       <c r="B82" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C82" s="0" t="s">
+      <c r="C82" s="3" t="s">
         <v>25</v>
       </c>
       <c r="D82" s="3" t="s">
@@ -2375,7 +2349,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="3" t="s">
         <v>53</v>
       </c>
@@ -2399,7 +2373,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
         <v>53</v>
       </c>
@@ -2423,14 +2397,14 @@
         <v>31</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="3" t="s">
         <v>53</v>
       </c>
       <c r="B85" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C85" s="9" t="s">
+      <c r="C85" s="3" t="s">
         <v>32</v>
       </c>
       <c r="D85" s="3" t="s">
@@ -2447,17 +2421,17 @@
         <v>31</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="0" t="s">
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B86" s="1" t="n">
+      <c r="B86" s="4" t="n">
         <v>4</v>
       </c>
       <c r="C86" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D86" s="0" t="s">
+      <c r="D86" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E86" s="3" t="str">
@@ -2472,16 +2446,16 @@
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="0" t="s">
+      <c r="A87" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B87" s="1" t="n">
+      <c r="B87" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C87" s="8" t="s">
+      <c r="C87" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D87" s="0" t="s">
+      <c r="D87" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E87" s="3" t="str">
@@ -2495,17 +2469,17 @@
         <v>36</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="0" t="s">
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B88" s="1" t="n">
+      <c r="B88" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C88" s="0" t="s">
+      <c r="C88" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D88" s="0" t="s">
+      <c r="D88" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E88" s="3" t="str">
@@ -2519,17 +2493,17 @@
         <v>50</v>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="0" t="s">
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B89" s="1" t="n">
+      <c r="B89" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C89" s="0" t="s">
+      <c r="C89" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D89" s="0" t="s">
+      <c r="D89" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E89" s="3" t="str">
@@ -2543,17 +2517,17 @@
         <v>34</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="0" t="s">
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B90" s="1" t="n">
+      <c r="B90" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C90" s="0" t="s">
+      <c r="C90" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D90" s="0" t="s">
+      <c r="D90" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E90" s="3" t="str">
@@ -2567,17 +2541,17 @@
         <v>20</v>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="0" t="s">
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B91" s="1" t="n">
+      <c r="B91" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C91" s="8" t="s">
+      <c r="C91" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D91" s="0" t="s">
+      <c r="D91" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E91" s="3" t="str">
@@ -2591,17 +2565,17 @@
         <v>22</v>
       </c>
     </row>
-    <row r="92" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="0" t="s">
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B92" s="1" t="n">
+      <c r="B92" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C92" s="0" t="s">
+      <c r="C92" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D92" s="0" t="s">
+      <c r="D92" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E92" s="3" t="str">
@@ -2615,17 +2589,17 @@
         <v>16</v>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="0" t="s">
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B93" s="1" t="n">
+      <c r="B93" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C93" s="0" t="s">
+      <c r="C93" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D93" s="0" t="s">
+      <c r="D93" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E93" s="3" t="str">
@@ -2639,17 +2613,17 @@
         <v>24</v>
       </c>
     </row>
-    <row r="94" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="0" t="s">
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B94" s="1" t="n">
+      <c r="B94" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C94" s="0" t="s">
+      <c r="C94" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D94" s="0" t="s">
+      <c r="D94" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E94" s="3" t="str">
@@ -2663,17 +2637,17 @@
         <v>26</v>
       </c>
     </row>
-    <row r="95" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="0" t="s">
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B95" s="1" t="n">
+      <c r="B95" s="4" t="n">
         <v>4</v>
       </c>
       <c r="C95" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D95" s="0" t="s">
+      <c r="D95" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E95" s="3" t="str">
@@ -2687,17 +2661,17 @@
         <v>29</v>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="0" t="s">
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B96" s="1" t="n">
+      <c r="B96" s="4" t="n">
         <v>4</v>
       </c>
       <c r="C96" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D96" s="0" t="s">
+      <c r="D96" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E96" s="3" t="str">
@@ -2711,17 +2685,17 @@
         <v>31</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="0" t="s">
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B97" s="1" t="n">
+      <c r="B97" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C97" s="9" t="s">
+      <c r="C97" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D97" s="0" t="s">
+      <c r="D97" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E97" s="3" t="str">
@@ -2735,7 +2709,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
         <v>54</v>
       </c>
@@ -2766,7 +2740,7 @@
       <c r="B99" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C99" s="8" t="s">
+      <c r="C99" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D99" s="3" t="s">
@@ -2783,14 +2757,14 @@
         <v>47</v>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="3" t="s">
         <v>55</v>
       </c>
       <c r="B100" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C100" s="0" t="s">
+      <c r="C100" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D100" s="3" t="s">
@@ -2807,14 +2781,14 @@
         <v>50</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="3" t="s">
         <v>55</v>
       </c>
       <c r="B101" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C101" s="0" t="s">
+      <c r="C101" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D101" s="3" t="s">
@@ -2831,14 +2805,14 @@
         <v>16</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="3" t="s">
         <v>55</v>
       </c>
       <c r="B102" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C102" s="0" t="s">
+      <c r="C102" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D102" s="3" t="s">
@@ -2855,14 +2829,14 @@
         <v>18</v>
       </c>
     </row>
-    <row r="103" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="3" t="s">
         <v>55</v>
       </c>
       <c r="B103" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C103" s="8" t="s">
+      <c r="C103" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D103" s="3" t="s">
@@ -2879,14 +2853,14 @@
         <v>20</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="3" t="s">
         <v>56</v>
       </c>
       <c r="B104" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C104" s="0" t="s">
+      <c r="C104" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D104" s="3" t="s">
@@ -2903,14 +2877,14 @@
         <v>22</v>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="3" t="s">
         <v>57</v>
       </c>
       <c r="B105" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C105" s="0" t="s">
+      <c r="C105" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D105" s="3" t="s">
@@ -2927,14 +2901,14 @@
         <v>58</v>
       </c>
     </row>
-    <row r="106" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="106" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="3" t="s">
         <v>54</v>
       </c>
       <c r="B106" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C106" s="0" t="s">
+      <c r="C106" s="3" t="s">
         <v>25</v>
       </c>
       <c r="D106" s="3" t="s">
@@ -2951,7 +2925,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="107" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="3" t="s">
         <v>57</v>
       </c>
@@ -2975,7 +2949,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="3" t="s">
         <v>57</v>
       </c>
@@ -2999,14 +2973,14 @@
         <v>58</v>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="3" t="s">
         <v>57</v>
       </c>
       <c r="B109" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C109" s="9" t="s">
+      <c r="C109" s="3" t="s">
         <v>32</v>
       </c>
       <c r="D109" s="3" t="s">
@@ -3023,17 +2997,17 @@
         <v>58</v>
       </c>
     </row>
-    <row r="110" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="0" t="s">
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B110" s="1" t="n">
+      <c r="B110" s="4" t="n">
         <v>5</v>
       </c>
       <c r="C110" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D110" s="0" t="s">
+      <c r="D110" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E110" s="3" t="str">
@@ -3048,16 +3022,16 @@
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="0" t="s">
+      <c r="A111" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B111" s="1" t="n">
+      <c r="B111" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C111" s="8" t="s">
+      <c r="C111" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D111" s="0" t="s">
+      <c r="D111" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E111" s="3" t="str">
@@ -3071,17 +3045,17 @@
         <v>47</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="0" t="s">
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B112" s="1" t="n">
+      <c r="B112" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C112" s="0" t="s">
+      <c r="C112" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D112" s="0" t="s">
+      <c r="D112" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E112" s="3" t="str">
@@ -3095,17 +3069,17 @@
         <v>50</v>
       </c>
     </row>
-    <row r="113" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="0" t="s">
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B113" s="1" t="n">
+      <c r="B113" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C113" s="0" t="s">
+      <c r="C113" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D113" s="0" t="s">
+      <c r="D113" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E113" s="3" t="str">
@@ -3119,17 +3093,17 @@
         <v>34</v>
       </c>
     </row>
-    <row r="114" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="0" t="s">
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B114" s="1" t="n">
+      <c r="B114" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C114" s="0" t="s">
+      <c r="C114" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D114" s="0" t="s">
+      <c r="D114" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E114" s="3" t="str">
@@ -3143,17 +3117,17 @@
         <v>20</v>
       </c>
     </row>
-    <row r="115" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="0" t="s">
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B115" s="1" t="n">
+      <c r="B115" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C115" s="8" t="s">
+      <c r="C115" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D115" s="0" t="s">
+      <c r="D115" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E115" s="3" t="str">
@@ -3167,17 +3141,17 @@
         <v>22</v>
       </c>
     </row>
-    <row r="116" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="0" t="s">
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B116" s="1" t="n">
+      <c r="B116" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C116" s="0" t="s">
+      <c r="C116" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D116" s="0" t="s">
+      <c r="D116" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E116" s="3" t="str">
@@ -3191,17 +3165,17 @@
         <v>16</v>
       </c>
     </row>
-    <row r="117" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="0" t="s">
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B117" s="1" t="n">
+      <c r="B117" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C117" s="0" t="s">
+      <c r="C117" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D117" s="0" t="s">
+      <c r="D117" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E117" s="3" t="str">
@@ -3215,17 +3189,17 @@
         <v>58</v>
       </c>
     </row>
-    <row r="118" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="0" t="s">
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B118" s="1" t="n">
+      <c r="B118" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C118" s="0" t="s">
+      <c r="C118" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D118" s="0" t="s">
+      <c r="D118" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E118" s="3" t="str">
@@ -3239,17 +3213,17 @@
         <v>26</v>
       </c>
     </row>
-    <row r="119" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="0" t="s">
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B119" s="1" t="n">
+      <c r="B119" s="4" t="n">
         <v>5</v>
       </c>
       <c r="C119" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D119" s="0" t="s">
+      <c r="D119" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E119" s="3" t="str">
@@ -3263,17 +3237,17 @@
         <v>58</v>
       </c>
     </row>
-    <row r="120" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="0" t="s">
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B120" s="1" t="n">
+      <c r="B120" s="4" t="n">
         <v>5</v>
       </c>
       <c r="C120" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D120" s="0" t="s">
+      <c r="D120" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E120" s="3" t="str">
@@ -3287,17 +3261,17 @@
         <v>58</v>
       </c>
     </row>
-    <row r="121" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A121" s="0" t="s">
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B121" s="1" t="n">
+      <c r="B121" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C121" s="9" t="s">
+      <c r="C121" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D121" s="0" t="s">
+      <c r="D121" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E121" s="3" t="str">
@@ -3311,7 +3285,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="122" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="122" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="3" t="s">
         <v>59</v>
       </c>
@@ -3342,7 +3316,7 @@
       <c r="B123" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C123" s="8" t="s">
+      <c r="C123" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D123" s="3" t="s">
@@ -3359,14 +3333,14 @@
         <v>47</v>
       </c>
     </row>
-    <row r="124" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="124" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="3" t="s">
         <v>46</v>
       </c>
       <c r="B124" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C124" s="0" t="s">
+      <c r="C124" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D124" s="3" t="s">
@@ -3383,14 +3357,14 @@
         <v>47</v>
       </c>
     </row>
-    <row r="125" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="125" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="3" t="s">
         <v>46</v>
       </c>
       <c r="B125" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C125" s="0" t="s">
+      <c r="C125" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D125" s="3" t="s">
@@ -3407,14 +3381,14 @@
         <v>16</v>
       </c>
     </row>
-    <row r="126" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="126" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="3" t="s">
         <v>46</v>
       </c>
       <c r="B126" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C126" s="0" t="s">
+      <c r="C126" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D126" s="3" t="s">
@@ -3431,14 +3405,14 @@
         <v>18</v>
       </c>
     </row>
-    <row r="127" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="127" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="3" t="s">
         <v>46</v>
       </c>
       <c r="B127" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C127" s="8" t="s">
+      <c r="C127" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D127" s="3" t="s">
@@ -3455,14 +3429,14 @@
         <v>20</v>
       </c>
     </row>
-    <row r="128" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="128" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="3" t="s">
         <v>54</v>
       </c>
       <c r="B128" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C128" s="0" t="s">
+      <c r="C128" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D128" s="3" t="s">
@@ -3479,14 +3453,14 @@
         <v>22</v>
       </c>
     </row>
-    <row r="129" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="129" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="3" t="s">
         <v>60</v>
       </c>
       <c r="B129" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C129" s="0" t="s">
+      <c r="C129" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D129" s="3" t="s">
@@ -3503,14 +3477,14 @@
         <v>61</v>
       </c>
     </row>
-    <row r="130" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="130" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="3" t="s">
         <v>57</v>
       </c>
       <c r="B130" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C130" s="0" t="s">
+      <c r="C130" s="3" t="s">
         <v>25</v>
       </c>
       <c r="D130" s="3" t="s">
@@ -3527,7 +3501,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="131" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="131" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="3" t="s">
         <v>62</v>
       </c>
@@ -3551,7 +3525,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="132" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="132" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="3" t="s">
         <v>62</v>
       </c>
@@ -3575,14 +3549,14 @@
         <v>31</v>
       </c>
     </row>
-    <row r="133" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="133" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="3" t="s">
         <v>62</v>
       </c>
       <c r="B133" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C133" s="9" t="s">
+      <c r="C133" s="3" t="s">
         <v>32</v>
       </c>
       <c r="D133" s="3" t="s">
@@ -3599,17 +3573,17 @@
         <v>31</v>
       </c>
     </row>
-    <row r="134" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A134" s="0" t="s">
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B134" s="1" t="n">
+      <c r="B134" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C134" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D134" s="0" t="s">
+      <c r="D134" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E134" s="3" t="str">
@@ -3624,16 +3598,16 @@
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A135" s="0" t="s">
+      <c r="A135" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B135" s="1" t="n">
+      <c r="B135" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C135" s="8" t="s">
+      <c r="C135" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D135" s="0" t="s">
+      <c r="D135" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E135" s="3" t="str">
@@ -3647,17 +3621,17 @@
         <v>47</v>
       </c>
     </row>
-    <row r="136" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A136" s="0" t="s">
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B136" s="1" t="n">
+      <c r="B136" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C136" s="0" t="s">
+      <c r="C136" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D136" s="0" t="s">
+      <c r="D136" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E136" s="3" t="str">
@@ -3671,17 +3645,17 @@
         <v>47</v>
       </c>
     </row>
-    <row r="137" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A137" s="0" t="s">
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B137" s="1" t="n">
+      <c r="B137" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C137" s="0" t="s">
+      <c r="C137" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D137" s="0" t="s">
+      <c r="D137" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E137" s="3" t="str">
@@ -3695,17 +3669,17 @@
         <v>34</v>
       </c>
     </row>
-    <row r="138" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A138" s="0" t="s">
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B138" s="1" t="n">
+      <c r="B138" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C138" s="0" t="s">
+      <c r="C138" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D138" s="0" t="s">
+      <c r="D138" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E138" s="3" t="str">
@@ -3719,17 +3693,17 @@
         <v>20</v>
       </c>
     </row>
-    <row r="139" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A139" s="0" t="s">
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B139" s="1" t="n">
+      <c r="B139" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C139" s="8" t="s">
+      <c r="C139" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D139" s="0" t="s">
+      <c r="D139" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E139" s="3" t="str">
@@ -3743,17 +3717,17 @@
         <v>22</v>
       </c>
     </row>
-    <row r="140" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A140" s="0" t="s">
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B140" s="1" t="n">
+      <c r="B140" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C140" s="0" t="s">
+      <c r="C140" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D140" s="0" t="s">
+      <c r="D140" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E140" s="3" t="str">
@@ -3767,17 +3741,17 @@
         <v>16</v>
       </c>
     </row>
-    <row r="141" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A141" s="0" t="s">
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A141" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B141" s="1" t="n">
+      <c r="B141" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C141" s="0" t="s">
+      <c r="C141" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D141" s="0" t="s">
+      <c r="D141" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E141" s="3" t="str">
@@ -3791,17 +3765,17 @@
         <v>61</v>
       </c>
     </row>
-    <row r="142" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A142" s="0" t="s">
+    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B142" s="1" t="n">
+      <c r="B142" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C142" s="0" t="s">
+      <c r="C142" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D142" s="0" t="s">
+      <c r="D142" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E142" s="3" t="str">
@@ -3815,17 +3789,17 @@
         <v>58</v>
       </c>
     </row>
-    <row r="143" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A143" s="0" t="s">
+    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B143" s="1" t="n">
+      <c r="B143" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C143" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D143" s="0" t="s">
+      <c r="D143" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E143" s="3" t="str">
@@ -3839,17 +3813,17 @@
         <v>29</v>
       </c>
     </row>
-    <row r="144" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A144" s="0" t="s">
+    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A144" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B144" s="1" t="n">
+      <c r="B144" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C144" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D144" s="0" t="s">
+      <c r="D144" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E144" s="3" t="str">
@@ -3863,17 +3837,17 @@
         <v>31</v>
       </c>
     </row>
-    <row r="145" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A145" s="0" t="s">
+    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A145" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B145" s="1" t="n">
+      <c r="B145" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C145" s="9" t="s">
+      <c r="C145" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D145" s="0" t="s">
+      <c r="D145" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E145" s="3" t="str">
@@ -3887,7 +3861,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="146" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="146" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="3" t="s">
         <v>63</v>
       </c>
@@ -3918,7 +3892,7 @@
       <c r="B147" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C147" s="8" t="s">
+      <c r="C147" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D147" s="3" t="s">
@@ -3935,14 +3909,14 @@
         <v>64</v>
       </c>
     </row>
-    <row r="148" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="148" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="3" t="s">
         <v>54</v>
       </c>
       <c r="B148" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C148" s="0" t="s">
+      <c r="C148" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D148" s="3" t="s">
@@ -3959,14 +3933,14 @@
         <v>47</v>
       </c>
     </row>
-    <row r="149" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="149" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="3" t="s">
         <v>54</v>
       </c>
       <c r="B149" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C149" s="0" t="s">
+      <c r="C149" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D149" s="3" t="s">
@@ -3983,14 +3957,14 @@
         <v>16</v>
       </c>
     </row>
-    <row r="150" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="150" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="3" t="s">
         <v>54</v>
       </c>
       <c r="B150" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C150" s="0" t="s">
+      <c r="C150" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D150" s="3" t="s">
@@ -4007,14 +3981,14 @@
         <v>18</v>
       </c>
     </row>
-    <row r="151" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="151" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="3" t="s">
         <v>54</v>
       </c>
       <c r="B151" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C151" s="8" t="s">
+      <c r="C151" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D151" s="3" t="s">
@@ -4031,14 +4005,14 @@
         <v>20</v>
       </c>
     </row>
-    <row r="152" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="152" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="3" t="s">
         <v>65</v>
       </c>
       <c r="B152" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C152" s="0" t="s">
+      <c r="C152" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D152" s="3" t="s">
@@ -4055,14 +4029,14 @@
         <v>58</v>
       </c>
     </row>
-    <row r="153" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="153" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="3" t="s">
         <v>62</v>
       </c>
       <c r="B153" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C153" s="0" t="s">
+      <c r="C153" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D153" s="3" t="s">
@@ -4079,14 +4053,14 @@
         <v>11</v>
       </c>
     </row>
-    <row r="154" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="154" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="3" t="s">
         <v>60</v>
       </c>
       <c r="B154" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C154" s="0" t="s">
+      <c r="C154" s="3" t="s">
         <v>25</v>
       </c>
       <c r="D154" s="3" t="s">
@@ -4103,7 +4077,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="155" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="155" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="3" t="s">
         <v>60</v>
       </c>
@@ -4127,7 +4101,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="156" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="156" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="3" t="s">
         <v>60</v>
       </c>
@@ -4151,14 +4125,14 @@
         <v>67</v>
       </c>
     </row>
-    <row r="157" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="157" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="3" t="s">
         <v>60</v>
       </c>
       <c r="B157" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C157" s="9" t="s">
+      <c r="C157" s="3" t="s">
         <v>32</v>
       </c>
       <c r="D157" s="3" t="s">
@@ -4175,17 +4149,17 @@
         <v>67</v>
       </c>
     </row>
-    <row r="158" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A158" s="0" t="s">
+    <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A158" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B158" s="1" t="n">
+      <c r="B158" s="4" t="n">
         <v>7</v>
       </c>
       <c r="C158" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D158" s="0" t="s">
+      <c r="D158" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E158" s="3" t="str">
@@ -4200,16 +4174,16 @@
       </c>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A159" s="0" t="s">
+      <c r="A159" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B159" s="1" t="n">
+      <c r="B159" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C159" s="8" t="s">
+      <c r="C159" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D159" s="0" t="s">
+      <c r="D159" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E159" s="3" t="str">
@@ -4223,17 +4197,17 @@
         <v>64</v>
       </c>
     </row>
-    <row r="160" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A160" s="0" t="s">
+    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A160" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B160" s="1" t="n">
+      <c r="B160" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C160" s="0" t="s">
+      <c r="C160" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D160" s="0" t="s">
+      <c r="D160" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E160" s="3" t="str">
@@ -4247,17 +4221,17 @@
         <v>47</v>
       </c>
     </row>
-    <row r="161" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A161" s="0" t="s">
+    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A161" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B161" s="1" t="n">
+      <c r="B161" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C161" s="0" t="s">
+      <c r="C161" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D161" s="0" t="s">
+      <c r="D161" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E161" s="3" t="str">
@@ -4271,17 +4245,17 @@
         <v>34</v>
       </c>
     </row>
-    <row r="162" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A162" s="0" t="s">
+    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A162" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B162" s="1" t="n">
+      <c r="B162" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C162" s="0" t="s">
+      <c r="C162" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D162" s="0" t="s">
+      <c r="D162" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E162" s="3" t="str">
@@ -4295,17 +4269,17 @@
         <v>20</v>
       </c>
     </row>
-    <row r="163" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A163" s="0" t="s">
+    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A163" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B163" s="1" t="n">
+      <c r="B163" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C163" s="8" t="s">
+      <c r="C163" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D163" s="0" t="s">
+      <c r="D163" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E163" s="3" t="str">
@@ -4319,17 +4293,17 @@
         <v>22</v>
       </c>
     </row>
-    <row r="164" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A164" s="0" t="s">
+    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A164" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B164" s="1" t="n">
+      <c r="B164" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C164" s="0" t="s">
+      <c r="C164" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D164" s="0" t="s">
+      <c r="D164" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E164" s="3" t="str">
@@ -4343,17 +4317,17 @@
         <v>58</v>
       </c>
     </row>
-    <row r="165" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A165" s="0" t="s">
+    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A165" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B165" s="1" t="n">
+      <c r="B165" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C165" s="0" t="s">
+      <c r="C165" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D165" s="0" t="s">
+      <c r="D165" s="3" t="s">
         <v>66</v>
       </c>
       <c r="E165" s="3" t="str">
@@ -4367,17 +4341,17 @@
         <v>24</v>
       </c>
     </row>
-    <row r="166" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A166" s="0" t="s">
+    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A166" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B166" s="1" t="n">
+      <c r="B166" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C166" s="0" t="s">
+      <c r="C166" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D166" s="0" t="s">
+      <c r="D166" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E166" s="3" t="str">
@@ -4391,17 +4365,17 @@
         <v>61</v>
       </c>
     </row>
-    <row r="167" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A167" s="0" t="s">
+    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A167" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B167" s="1" t="n">
+      <c r="B167" s="4" t="n">
         <v>7</v>
       </c>
       <c r="C167" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D167" s="0" t="s">
+      <c r="D167" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E167" s="3" t="str">
@@ -4415,17 +4389,17 @@
         <v>67</v>
       </c>
     </row>
-    <row r="168" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A168" s="0" t="s">
+    <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A168" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B168" s="1" t="n">
+      <c r="B168" s="4" t="n">
         <v>7</v>
       </c>
       <c r="C168" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D168" s="0" t="s">
+      <c r="D168" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E168" s="3" t="str">
@@ -4439,17 +4413,17 @@
         <v>67</v>
       </c>
     </row>
-    <row r="169" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A169" s="0" t="s">
+    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A169" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B169" s="1" t="n">
+      <c r="B169" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C169" s="9" t="s">
+      <c r="C169" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D169" s="0" t="s">
+      <c r="D169" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E169" s="3" t="str">
@@ -4463,7 +4437,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="170" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="170" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="3" t="s">
         <v>57</v>
       </c>
@@ -4494,7 +4468,7 @@
       <c r="B171" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="C171" s="8" t="s">
+      <c r="C171" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D171" s="3" t="s">
@@ -4511,14 +4485,14 @@
         <v>58</v>
       </c>
     </row>
-    <row r="172" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="172" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="3" t="s">
         <v>63</v>
       </c>
       <c r="B172" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="C172" s="0" t="s">
+      <c r="C172" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D172" s="3" t="s">
@@ -4535,14 +4509,14 @@
         <v>64</v>
       </c>
     </row>
-    <row r="173" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="173" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="3" t="s">
         <v>65</v>
       </c>
       <c r="B173" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="C173" s="0" t="s">
+      <c r="C173" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D173" s="3" t="s">
@@ -4559,14 +4533,14 @@
         <v>58</v>
       </c>
     </row>
-    <row r="174" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="174" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="3" t="s">
         <v>65</v>
       </c>
       <c r="B174" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="C174" s="0" t="s">
+      <c r="C174" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D174" s="3" t="s">
@@ -4583,14 +4557,14 @@
         <v>58</v>
       </c>
     </row>
-    <row r="175" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="175" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="3" t="s">
         <v>65</v>
       </c>
       <c r="B175" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="C175" s="8" t="s">
+      <c r="C175" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D175" s="3" t="s">
@@ -4607,14 +4581,14 @@
         <v>58</v>
       </c>
     </row>
-    <row r="176" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="176" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="3" t="s">
         <v>60</v>
       </c>
       <c r="B176" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="C176" s="0" t="s">
+      <c r="C176" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D176" s="3" t="s">
@@ -4631,14 +4605,14 @@
         <v>61</v>
       </c>
     </row>
-    <row r="177" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="177" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="3" t="s">
         <v>68</v>
       </c>
       <c r="B177" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="C177" s="0" t="s">
+      <c r="C177" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D177" s="3" t="s">
@@ -4655,14 +4629,14 @@
         <v>64</v>
       </c>
     </row>
-    <row r="178" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="178" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="3" t="s">
         <v>62</v>
       </c>
       <c r="B178" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="C178" s="0" t="s">
+      <c r="C178" s="3" t="s">
         <v>25</v>
       </c>
       <c r="D178" s="3" t="s">
@@ -4679,24 +4653,24 @@
         <v>11</v>
       </c>
     </row>
-    <row r="179" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A179" s="0" t="s">
+    <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A179" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B179" s="1" t="n">
+      <c r="B179" s="4" t="n">
         <v>8</v>
       </c>
       <c r="C179" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D179" s="0" t="s">
+      <c r="D179" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E179" s="3" t="str">
         <f aca="false">_xlfn.CONCAT("Curso de ",A179," de tipo ",D179, " para ",C179," durante el ciclo escolar ", F179,".")</f>
         <v>Curso de Artes de tipo Formativo para SECUNDARIA_3 durante el ciclo escolar CE20212022.</v>
       </c>
-      <c r="F179" s="0" t="s">
+      <c r="F179" s="3" t="s">
         <v>33</v>
       </c>
       <c r="G179" s="2" t="s">
@@ -4704,16 +4678,16 @@
       </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A180" s="0" t="s">
+      <c r="A180" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B180" s="1" t="n">
+      <c r="B180" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="C180" s="8" t="s">
+      <c r="C180" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D180" s="0" t="s">
+      <c r="D180" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E180" s="3" t="str">
@@ -4727,17 +4701,17 @@
         <v>58</v>
       </c>
     </row>
-    <row r="181" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A181" s="0" t="s">
+    <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A181" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B181" s="1" t="n">
+      <c r="B181" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="C181" s="0" t="s">
+      <c r="C181" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D181" s="0" t="s">
+      <c r="D181" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E181" s="3" t="str">
@@ -4751,17 +4725,17 @@
         <v>64</v>
       </c>
     </row>
-    <row r="182" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A182" s="0" t="s">
+    <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A182" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B182" s="1" t="n">
+      <c r="B182" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="C182" s="0" t="s">
+      <c r="C182" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D182" s="0" t="s">
+      <c r="D182" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E182" s="3" t="str">
@@ -4775,17 +4749,17 @@
         <v>58</v>
       </c>
     </row>
-    <row r="183" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A183" s="0" t="s">
+    <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A183" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B183" s="1" t="n">
+      <c r="B183" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="C183" s="0" t="s">
+      <c r="C183" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D183" s="0" t="s">
+      <c r="D183" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E183" s="3" t="str">
@@ -4799,17 +4773,17 @@
         <v>58</v>
       </c>
     </row>
-    <row r="184" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A184" s="0" t="s">
+    <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A184" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B184" s="1" t="n">
+      <c r="B184" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="C184" s="8" t="s">
+      <c r="C184" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D184" s="0" t="s">
+      <c r="D184" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E184" s="3" t="str">
@@ -4823,17 +4797,17 @@
         <v>58</v>
       </c>
     </row>
-    <row r="185" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A185" s="0" t="s">
+    <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A185" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B185" s="1" t="n">
+      <c r="B185" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="C185" s="0" t="s">
+      <c r="C185" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D185" s="0" t="s">
+      <c r="D185" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E185" s="3" t="str">
@@ -4847,17 +4821,17 @@
         <v>61</v>
       </c>
     </row>
-    <row r="186" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A186" s="0" t="s">
+    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A186" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B186" s="1" t="n">
+      <c r="B186" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="C186" s="0" t="s">
+      <c r="C186" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D186" s="0" t="s">
+      <c r="D186" s="3" t="s">
         <v>66</v>
       </c>
       <c r="E186" s="3" t="str">
@@ -4871,17 +4845,17 @@
         <v>64</v>
       </c>
     </row>
-    <row r="187" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A187" s="0" t="s">
+    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A187" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B187" s="1" t="n">
+      <c r="B187" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="C187" s="0" t="s">
+      <c r="C187" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D187" s="0" t="s">
+      <c r="D187" s="3" t="s">
         <v>66</v>
       </c>
       <c r="E187" s="3" t="str">
@@ -4895,7 +4869,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="188" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="188" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="3" t="s">
         <v>60</v>
       </c>
@@ -4926,7 +4900,7 @@
       <c r="B189" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="C189" s="8" t="s">
+      <c r="C189" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D189" s="3" t="s">
@@ -4943,14 +4917,14 @@
         <v>67</v>
       </c>
     </row>
-    <row r="190" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="190" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="3" t="s">
         <v>57</v>
       </c>
       <c r="B190" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="C190" s="0" t="s">
+      <c r="C190" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D190" s="3" t="s">
@@ -4967,14 +4941,14 @@
         <v>58</v>
       </c>
     </row>
-    <row r="191" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="191" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="3" t="s">
         <v>60</v>
       </c>
       <c r="B191" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="C191" s="0" t="s">
+      <c r="C191" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D191" s="3" t="s">
@@ -4991,14 +4965,14 @@
         <v>61</v>
       </c>
     </row>
-    <row r="192" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="192" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="3" t="s">
         <v>60</v>
       </c>
       <c r="B192" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="C192" s="0" t="s">
+      <c r="C192" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D192" s="3" t="s">
@@ -5015,14 +4989,14 @@
         <v>61</v>
       </c>
     </row>
-    <row r="193" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="193" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="3" t="s">
         <v>60</v>
       </c>
       <c r="B193" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="C193" s="8" t="s">
+      <c r="C193" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D193" s="3" t="s">
@@ -5039,14 +5013,14 @@
         <v>61</v>
       </c>
     </row>
-    <row r="194" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="194" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="3" t="s">
         <v>69</v>
       </c>
       <c r="B194" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="C194" s="0" t="s">
+      <c r="C194" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D194" s="3" t="s">
@@ -5063,14 +5037,14 @@
         <v>11</v>
       </c>
     </row>
-    <row r="195" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="195" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="3" t="s">
         <v>68</v>
       </c>
       <c r="B195" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="C195" s="0" t="s">
+      <c r="C195" s="3" t="s">
         <v>25</v>
       </c>
       <c r="D195" s="3" t="s">
@@ -5087,17 +5061,17 @@
         <v>64</v>
       </c>
     </row>
-    <row r="196" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A196" s="0" t="s">
+    <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A196" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B196" s="1" t="n">
+      <c r="B196" s="4" t="n">
         <v>9</v>
       </c>
       <c r="C196" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D196" s="0" t="s">
+      <c r="D196" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E196" s="3" t="str">
@@ -5112,16 +5086,16 @@
       </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A197" s="0" t="s">
+      <c r="A197" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B197" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="C197" s="8" t="s">
+      <c r="B197" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C197" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D197" s="0" t="s">
+      <c r="D197" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E197" s="3" t="str">
@@ -5135,17 +5109,17 @@
         <v>67</v>
       </c>
     </row>
-    <row r="198" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A198" s="0" t="s">
+    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A198" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B198" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="C198" s="0" t="s">
+      <c r="B198" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C198" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D198" s="0" t="s">
+      <c r="D198" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E198" s="3" t="str">
@@ -5159,17 +5133,17 @@
         <v>58</v>
       </c>
     </row>
-    <row r="199" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A199" s="0" t="s">
+    <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A199" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B199" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="C199" s="0" t="s">
+      <c r="B199" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C199" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D199" s="0" t="s">
+      <c r="D199" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E199" s="3" t="str">
@@ -5183,17 +5157,17 @@
         <v>61</v>
       </c>
     </row>
-    <row r="200" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A200" s="0" t="s">
+    <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A200" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B200" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="C200" s="0" t="s">
+      <c r="B200" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C200" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D200" s="0" t="s">
+      <c r="D200" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E200" s="3" t="str">
@@ -5207,17 +5181,17 @@
         <v>61</v>
       </c>
     </row>
-    <row r="201" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A201" s="0" t="s">
+    <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A201" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B201" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="C201" s="8" t="s">
+      <c r="B201" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C201" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D201" s="0" t="s">
+      <c r="D201" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E201" s="3" t="str">
@@ -5231,17 +5205,17 @@
         <v>61</v>
       </c>
     </row>
-    <row r="202" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A202" s="0" t="s">
+    <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A202" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B202" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="C202" s="0" t="s">
+      <c r="B202" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C202" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D202" s="0" t="s">
+      <c r="D202" s="3" t="s">
         <v>66</v>
       </c>
       <c r="E202" s="3" t="str">
@@ -5255,17 +5229,17 @@
         <v>16</v>
       </c>
     </row>
-    <row r="203" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A203" s="0" t="s">
+    <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A203" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B203" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="C203" s="0" t="s">
+      <c r="B203" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C203" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D203" s="0" t="s">
+      <c r="D203" s="3" t="s">
         <v>66</v>
       </c>
       <c r="E203" s="3" t="str">
@@ -5279,7 +5253,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="204" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="204" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="3" t="s">
         <v>70</v>
       </c>
@@ -5310,7 +5284,7 @@
       <c r="B205" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="C205" s="8" t="s">
+      <c r="C205" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D205" s="3" t="s">
@@ -5327,14 +5301,14 @@
         <v>64</v>
       </c>
     </row>
-    <row r="206" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="206" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A206" s="3" t="s">
         <v>60</v>
       </c>
       <c r="B206" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="C206" s="0" t="s">
+      <c r="C206" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D206" s="3" t="s">
@@ -5351,14 +5325,14 @@
         <v>67</v>
       </c>
     </row>
-    <row r="207" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="207" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="3" t="s">
         <v>69</v>
       </c>
       <c r="B207" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="C207" s="0" t="s">
+      <c r="C207" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D207" s="3" t="s">
@@ -5375,14 +5349,14 @@
         <v>11</v>
       </c>
     </row>
-    <row r="208" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="208" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="3" t="s">
         <v>69</v>
       </c>
       <c r="B208" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="C208" s="0" t="s">
+      <c r="C208" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D208" s="3" t="s">
@@ -5399,14 +5373,14 @@
         <v>11</v>
       </c>
     </row>
-    <row r="209" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="209" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="3" t="s">
         <v>69</v>
       </c>
       <c r="B209" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="C209" s="8" t="s">
+      <c r="C209" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D209" s="3" t="s">
@@ -5423,14 +5397,14 @@
         <v>11</v>
       </c>
     </row>
-    <row r="210" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="210" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="3" t="s">
         <v>71</v>
       </c>
       <c r="B210" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="C210" s="0" t="s">
+      <c r="C210" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D210" s="3" t="s">
@@ -5447,17 +5421,17 @@
         <v>64</v>
       </c>
     </row>
-    <row r="211" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A211" s="0" t="s">
+    <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A211" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B211" s="1" t="n">
+      <c r="B211" s="4" t="n">
         <v>10</v>
       </c>
       <c r="C211" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D211" s="0" t="s">
+      <c r="D211" s="3" t="s">
         <v>66</v>
       </c>
       <c r="E211" s="3" t="str">
@@ -5472,16 +5446,16 @@
       </c>
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A212" s="0" t="s">
+      <c r="A212" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B212" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="C212" s="8" t="s">
+      <c r="B212" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C212" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D212" s="0" t="s">
+      <c r="D212" s="3" t="s">
         <v>66</v>
       </c>
       <c r="E212" s="3" t="str">
@@ -5495,17 +5469,17 @@
         <v>64</v>
       </c>
     </row>
-    <row r="213" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A213" s="0" t="s">
+    <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A213" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B213" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="C213" s="0" t="s">
+      <c r="B213" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C213" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D213" s="0" t="s">
+      <c r="D213" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E213" s="3" t="str">
@@ -5519,17 +5493,17 @@
         <v>67</v>
       </c>
     </row>
-    <row r="214" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A214" s="0" t="s">
+    <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A214" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B214" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="C214" s="0" t="s">
+      <c r="B214" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C214" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D214" s="0" t="s">
+      <c r="D214" s="3" t="s">
         <v>66</v>
       </c>
       <c r="E214" s="3" t="str">
@@ -5543,17 +5517,17 @@
         <v>11</v>
       </c>
     </row>
-    <row r="215" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A215" s="0" t="s">
+    <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A215" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B215" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="C215" s="0" t="s">
+      <c r="B215" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C215" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D215" s="0" t="s">
+      <c r="D215" s="3" t="s">
         <v>66</v>
       </c>
       <c r="E215" s="3" t="str">
@@ -5567,17 +5541,17 @@
         <v>11</v>
       </c>
     </row>
-    <row r="216" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A216" s="0" t="s">
+    <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A216" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B216" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="C216" s="8" t="s">
+      <c r="B216" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C216" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D216" s="0" t="s">
+      <c r="D216" s="3" t="s">
         <v>66</v>
       </c>
       <c r="E216" s="3" t="str">
@@ -5591,17 +5565,17 @@
         <v>22</v>
       </c>
     </row>
-    <row r="217" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A217" s="0" t="s">
+    <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A217" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B217" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="C217" s="0" t="s">
+      <c r="B217" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C217" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D217" s="0" t="s">
+      <c r="D217" s="3" t="s">
         <v>66</v>
       </c>
       <c r="E217" s="3" t="str">
@@ -5615,7 +5589,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="218" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="218" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="3" t="s">
         <v>72</v>
       </c>
@@ -5646,7 +5620,7 @@
       <c r="B219" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="C219" s="8" t="s">
+      <c r="C219" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D219" s="3" t="s">
@@ -5663,14 +5637,14 @@
         <v>50</v>
       </c>
     </row>
-    <row r="220" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="220" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="3" t="s">
         <v>70</v>
       </c>
       <c r="B220" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="C220" s="0" t="s">
+      <c r="C220" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D220" s="3" t="s">
@@ -5687,14 +5661,14 @@
         <v>64</v>
       </c>
     </row>
-    <row r="221" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="221" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="3" t="s">
         <v>71</v>
       </c>
       <c r="B221" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="C221" s="0" t="s">
+      <c r="C221" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D221" s="3" t="s">
@@ -5711,14 +5685,14 @@
         <v>64</v>
       </c>
     </row>
-    <row r="222" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="222" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="3" t="s">
         <v>71</v>
       </c>
       <c r="B222" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="C222" s="0" t="s">
+      <c r="C222" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D222" s="3" t="s">
@@ -5735,14 +5709,14 @@
         <v>64</v>
       </c>
     </row>
-    <row r="223" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="223" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="3" t="s">
         <v>71</v>
       </c>
       <c r="B223" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="C223" s="8" t="s">
+      <c r="C223" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D223" s="3" t="s">
@@ -5759,17 +5733,17 @@
         <v>64</v>
       </c>
     </row>
-    <row r="224" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A224" s="0" t="s">
+    <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A224" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B224" s="1" t="n">
+      <c r="B224" s="4" t="n">
         <v>11</v>
       </c>
       <c r="C224" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D224" s="0" t="s">
+      <c r="D224" s="3" t="s">
         <v>66</v>
       </c>
       <c r="E224" s="3" t="str">
@@ -5784,16 +5758,16 @@
       </c>
     </row>
     <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A225" s="0" t="s">
+      <c r="A225" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B225" s="1" t="n">
+      <c r="B225" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="C225" s="8" t="s">
+      <c r="C225" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D225" s="0" t="s">
+      <c r="D225" s="3" t="s">
         <v>66</v>
       </c>
       <c r="E225" s="3" t="str">
@@ -5807,17 +5781,17 @@
         <v>50</v>
       </c>
     </row>
-    <row r="226" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A226" s="0" t="s">
+    <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A226" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B226" s="1" t="n">
+      <c r="B226" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="C226" s="0" t="s">
+      <c r="C226" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D226" s="0" t="s">
+      <c r="D226" s="3" t="s">
         <v>66</v>
       </c>
       <c r="E226" s="3" t="str">
@@ -5831,17 +5805,17 @@
         <v>64</v>
       </c>
     </row>
-    <row r="227" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A227" s="0" t="s">
+    <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A227" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B227" s="1" t="n">
+      <c r="B227" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="C227" s="0" t="s">
+      <c r="C227" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D227" s="0" t="s">
+      <c r="D227" s="3" t="s">
         <v>66</v>
       </c>
       <c r="E227" s="3" t="str">
@@ -5855,17 +5829,17 @@
         <v>64</v>
       </c>
     </row>
-    <row r="228" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A228" s="0" t="s">
+    <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A228" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B228" s="1" t="n">
+      <c r="B228" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="C228" s="0" t="s">
+      <c r="C228" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D228" s="0" t="s">
+      <c r="D228" s="3" t="s">
         <v>66</v>
       </c>
       <c r="E228" s="3" t="str">
@@ -5879,17 +5853,17 @@
         <v>64</v>
       </c>
     </row>
-    <row r="229" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A229" s="0" t="s">
+    <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A229" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B229" s="1" t="n">
+      <c r="B229" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="C229" s="8" t="s">
+      <c r="C229" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D229" s="0" t="s">
+      <c r="D229" s="3" t="s">
         <v>66</v>
       </c>
       <c r="E229" s="3" t="str">
@@ -5903,14 +5877,14 @@
         <v>64</v>
       </c>
     </row>
-    <row r="230" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="230" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B230" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="C230" s="0" t="s">
+      <c r="C230" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D230" s="3" t="s">
@@ -5927,17 +5901,17 @@
         <v>50</v>
       </c>
     </row>
-    <row r="231" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A231" s="0" t="s">
+    <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A231" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B231" s="1" t="n">
+      <c r="B231" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="C231" s="0" t="s">
+      <c r="C231" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D231" s="0" t="s">
+      <c r="D231" s="3" t="s">
         <v>66</v>
       </c>
       <c r="E231" s="3" t="str">
@@ -5951,17 +5925,139 @@
         <v>50</v>
       </c>
     </row>
-    <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C233" s="3"/>
-    </row>
+    <row r="1048445" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048446" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048447" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048448" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048449" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048450" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048451" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048452" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048453" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048454" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048455" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048456" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048457" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048458" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048459" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048460" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048461" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048462" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048463" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048464" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048465" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048466" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048467" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048468" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048469" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048470" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048471" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048472" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048473" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048474" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048475" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048476" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048477" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048478" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048479" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048480" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048481" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048482" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048483" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048484" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048485" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048486" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048487" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048488" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048489" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048490" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048491" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048492" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048493" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048494" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048495" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048496" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048497" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048498" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048499" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048500" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048501" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048502" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048503" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048504" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048505" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048506" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048507" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048508" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048509" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048510" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048511" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048512" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048513" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048514" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048515" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048516" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048517" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048518" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048519" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048520" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048521" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048522" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048523" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048524" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048525" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048526" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048527" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048528" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048529" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048530" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048531" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048532" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048533" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048534" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048535" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048536" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048537" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048538" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048539" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048540" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048541" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048542" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048543" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048544" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048545" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048546" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048547" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048548" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048549" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048550" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048551" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048552" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048553" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048554" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048555" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <autoFilter ref="A1:G231">
-    <filterColumn colId="2">
-      <customFilters and="true">
-        <customFilter operator="equal" val="2° de Secundaria"/>
-      </customFilters>
-    </filterColumn>
-  </autoFilter>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511805555555555" footer="0.511805555555555"/>
   <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -5969,6 +6065,5 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>